<commit_message>
Update Phase 1 checklist from verification; keep audit tooling
</commit_message>
<xml_diff>
--- a/docs/SMF_Phase1_Functional_Compliance_Test_Checklist.xlsx
+++ b/docs/SMF_Phase1_Functional_Compliance_Test_Checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
   <si>
     <t>ID</t>
   </si>
@@ -473,6 +473,66 @@
   </si>
   <si>
     <t>Re-verification of the 30 Phase 1 findings: 11 confirmed FIXED (language switcher, social links, name split, upload 1MB cap, security headers, robots.txt, API 400 not 500, news thumbnails, community link, mobile country-code selector, unlinked pages [redirect to canonical]); 5 PARTIAL (calendar year-grid still broken, age auto-category, data-standards, server-side validation, athlete photos placeholders); 3 STILL OPEN (server banner on staging, Cloudflare/origin at launch, Try-Muaythai needs clubs); 11 pending live UI/admin verification. Status reflected in Websitelocal.xlsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar year-grid fixed: the grid used auto-fill and rendered 12 months across 5 ragged columns, and empty months stretched to full row height. Now a 4x3 quarter layout (3/2/1 at narrower widths) with compact empty months. Verified at 1440/900/480 in both AR/RTL and EN/LTR, no horizontal overflow, no console errors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List/grid toggle and year navigation verified working: 12 month cells, 34 events, year buttons plus 'All years'. Grid layout defect behind the earlier Fail is fixed. Verified in both languages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Athlete registration submits and is stored: POST /api/registrations returned a reference number (SMF-A-YYYY-NNNNN) and the record was retrievable from the admin queue with its payload and status. Verified on a local instance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All four types submit and store correctly, each with its own reference prefix: athlete (SMF-A), coach (SMF-T), referee (SMF-O), club (SMF-C). Each appears in the admin queue under the right type. Type-specific rules are enforced - referee grade, refereeing start date and tournament history for referees; applicant role, facility type, owner and head coach for clubs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submitted applications appear in the admin review queue with applicant name, contact, type, status, approval stage and their uploaded documents. The list projection deliberately omits the full payload so national ID, date of birth and guardian details are only loaded when a reviewer opens the record, and that access is itself audited.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full chain verified against the admin console: new -&gt; under review -&gt; awaiting completion -&gt; under review -&gt; awaiting approval -&gt; approved, plus suspend/reinstate and renewal. Illegal transitions are refused with 400 (e.g. new -&gt; approved directly) and each status requiring a reason is refused with 400 when it is missing. Verified on a local instance; re-run on the deployed environment when access is provided.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email and SMS are sent on every lifecycle event: submission (with reference number), completion request, acceptance, rejection (with reason), renewal, expiry, and suspension/cancellation. Verified via the outbox: 6 emails + 5 SMS across one request's lifecycle, Arabic rendered correctly with placeholders substituted. No SMTP or SMS gateway is configured yet, so messages are written to the outbox rather than delivered - that is configuration, not code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Server-side re-validation confirmed: posting directly to the API with client-valid data was rejected with 400 and per-field bilingual errors (required name parts, document type, age band, phone format). The admin edit endpoint re-validates with the same rules, so a correction cannot introduce data the public form would refuse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audit trail implemented and verified: actor, role, action, from/to status, timestamp and reason are recorded for every status change, edit, renewal, suspension, expiry, export, attachment view and deletion - including refused attempts (permission_denied). Entries are append-only and commit in the same transaction as the change they describe. Reasons are stored but field values are not, so the trail names what changed without copying applicant PII.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audited across 6 pages (home, calendar, results archive, contact, registration, news) against WCAG AA. Fixed: the selected view toggle on the results archive rendered white text on a white background (a specificity clash made the label invisible); section subtitles site-wide were 2.54:1; the IFMA source chip 2.93:1; gold and bronze medal badges 2.63:1 and 3.1:1. All now meet 4.5:1. Redundant unnamed image links removed from the accessibility tree. Verified clean: lang/dir set, one h1 per page with no skipped levels, &lt;main&gt; landmark, skip-to-content link, all images have alt, all form controls labelled, focus visible.</t>
   </si>
 </sst>
 </file>
@@ -986,10 +1046,10 @@
         <v>13</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>14</v>
+        <v>151</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1107,7 +1167,10 @@
         <v>35</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>14</v>
+        <v>153</v>
+      </c>
+      <c r="H7" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1225,7 +1288,10 @@
         <v>55</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>44</v>
+        <v>155</v>
+      </c>
+      <c r="H12" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -1248,7 +1314,10 @@
         <v>58</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>44</v>
+        <v>157</v>
+      </c>
+      <c r="H13" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1271,7 +1340,10 @@
         <v>61</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>44</v>
+        <v>159</v>
+      </c>
+      <c r="H14" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1294,7 +1366,10 @@
         <v>64</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>44</v>
+        <v>161</v>
+      </c>
+      <c r="H15" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1317,7 +1392,10 @@
         <v>67</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>44</v>
+        <v>163</v>
+      </c>
+      <c r="H16" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1412,7 +1490,10 @@
         <v>82</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>44</v>
+        <v>165</v>
+      </c>
+      <c r="H20" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
@@ -1694,7 +1775,10 @@
         <v>126</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>44</v>
+        <v>167</v>
+      </c>
+      <c r="H32" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1740,7 +1824,10 @@
         <v>134</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>135</v>
+        <v>169</v>
+      </c>
+      <c r="H34" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>